<commit_message>
Rehacer el formato de los siete documentos para que se puedan entregar.
Encabezados, filas alternadas y un dashboard con tarjetas y gráficas. El registro de ventas vuelve a incluir las filas que sí se leen en la foto.

Co-authored-by: sebsotoosolis-ui <sebsotoosolis-ui@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/documentos/Analisis de ventas.xlsx
+++ b/documentos/Analisis de ventas.xlsx
@@ -9,9 +9,7 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hoja1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Hoja1'!$A$1:$D$9</definedName>
-  </definedNames>
+  <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -19,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -31,15 +29,27 @@
       <name val="Calibri"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
+      <sz val="18"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
       <sz val="11"/>
     </font>
     <font>
       <name val="Calibri"/>
-      <color rgb="001A1A1A"/>
+      <color rgb="001F2933"/>
       <sz val="11"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001F4E79"/>
+      <sz val="16"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -48,12 +58,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="001B3A4B"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="001F4E79"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00D6E3F0"/>
+        <fgColor rgb="00E7F0F7"/>
       </patternFill>
     </fill>
     <fill>
@@ -61,8 +76,18 @@
         <fgColor rgb="00FFFFFF"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF3D6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFBF2"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -70,45 +95,50 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border/>
     <border>
       <left style="thin">
-        <color rgb="00B0B8C4"/>
+        <color rgb="00D5DEE7"/>
       </left>
       <right style="thin">
-        <color rgb="00B0B8C4"/>
+        <color rgb="00D5DEE7"/>
       </right>
       <top style="thin">
-        <color rgb="00B0B8C4"/>
+        <color rgb="00D5DEE7"/>
       </top>
       <bottom style="thin">
-        <color rgb="00B0B8C4"/>
+        <color rgb="00D5DEE7"/>
       </bottom>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="1" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="1" fontId="4" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="1" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="1" fontId="4" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -473,211 +503,217 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="001F4E79"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D9"/>
+  <dimension ref="A1:D11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="36" customWidth="1" min="1" max="1"/>
     <col width="28" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
     <col width="78" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1">
+    <row r="1" ht="38" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
+          <t>Análisis de ventas</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="n"/>
+      <c r="C1" s="2" t="n"/>
+      <c r="D1" s="2" t="n"/>
+    </row>
+    <row r="2" ht="10" customHeight="1"/>
+    <row r="3" ht="28" customHeight="1">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
           <t>Indicador</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B3" s="3" t="inlineStr">
         <is>
           <t>Fórmula</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C3" s="3" t="inlineStr">
         <is>
           <t>Resultado</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D3" s="3" t="inlineStr">
         <is>
           <t>Interpretación</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="22" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
+    <row r="4" ht="28" customHeight="1">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>Total de Ventas</t>
         </is>
       </c>
-      <c r="B2" s="3" t="inlineStr">
+      <c r="B4" s="5" t="inlineStr">
         <is>
           <t>CONTARA()</t>
         </is>
       </c>
-      <c r="C2" s="4" t="n">
+      <c r="C4" s="6" t="n">
         <v>40</v>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="D4" s="4" t="inlineStr">
         <is>
           <t>Cuenta todos los registros de ventas.</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="22" customHeight="1">
-      <c r="A3" s="5" t="inlineStr">
+    <row r="5" ht="28" customHeight="1">
+      <c r="A5" s="7" t="inlineStr">
         <is>
           <t>Ventas que alcanzaron meta</t>
         </is>
       </c>
-      <c r="B3" s="6" t="inlineStr">
+      <c r="B5" s="8" t="inlineStr">
         <is>
           <t>CONTAR.SI()</t>
         </is>
       </c>
-      <c r="C3" s="7" t="n">
+      <c r="C5" s="9" t="n">
         <v>26</v>
       </c>
-      <c r="D3" s="5" t="inlineStr">
+      <c r="D5" s="7" t="inlineStr">
         <is>
           <t>De las 40 ventas, 26 alcanzaron la meta establecida.</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="22" customHeight="1">
-      <c r="A4" s="2" t="inlineStr">
+    <row r="6" ht="28" customHeight="1">
+      <c r="A6" s="4" t="inlineStr">
         <is>
           <t>Ventas de Región Norte</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B6" s="5" t="inlineStr">
         <is>
           <t>CONTAR.SI()</t>
         </is>
       </c>
-      <c r="C4" s="4" t="n">
+      <c r="C6" s="6" t="n">
         <v>7</v>
       </c>
-      <c r="D4" s="2" t="inlineStr">
+      <c r="D6" s="4" t="inlineStr">
         <is>
           <t>De las 40 ventas, 7 pertenecen a la región Norte.</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="22" customHeight="1">
-      <c r="A5" s="5" t="inlineStr">
+    <row r="7" ht="28" customHeight="1">
+      <c r="A7" s="7" t="inlineStr">
         <is>
           <t>Ventas de laptop</t>
         </is>
       </c>
-      <c r="B5" s="6" t="inlineStr">
+      <c r="B7" s="8" t="inlineStr">
         <is>
           <t>CONTAR.SI()</t>
         </is>
       </c>
-      <c r="C5" s="7" t="n">
+      <c r="C7" s="9" t="n">
         <v>15</v>
       </c>
-      <c r="D5" s="5" t="inlineStr">
+      <c r="D7" s="7" t="inlineStr">
         <is>
           <t>De las 40 ventas, 15 corresponden al producto Laptop.</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="22" customHeight="1">
-      <c r="A6" s="2" t="inlineStr">
+    <row r="8" ht="28" customHeight="1">
+      <c r="A8" s="4" t="inlineStr">
         <is>
           <t>Ventas Excelentes</t>
         </is>
       </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="B8" s="5" t="inlineStr">
         <is>
           <t>CONTAR.SI()</t>
         </is>
       </c>
-      <c r="C6" s="4" t="n">
+      <c r="C8" s="6" t="n">
         <v>5</v>
       </c>
-      <c r="D6" s="2" t="inlineStr">
+      <c r="D8" s="4" t="inlineStr">
         <is>
           <t>Se registraron 5 ventas con una satisfacción de 95% o más.</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="22" customHeight="1">
-      <c r="A7" s="5" t="inlineStr">
+    <row r="9" ht="28" customHeight="1">
+      <c r="A9" s="7" t="inlineStr">
         <is>
           <t>Norte y meta cumplida</t>
         </is>
       </c>
-      <c r="B7" s="6" t="inlineStr">
+      <c r="B9" s="8" t="inlineStr">
         <is>
           <t>CONTAR.SI.CONJUNTO()</t>
         </is>
       </c>
-      <c r="C7" s="7" t="n">
+      <c r="C9" s="9" t="n">
         <v>6</v>
       </c>
-      <c r="D7" s="5" t="inlineStr">
+      <c r="D9" s="7" t="inlineStr">
         <is>
           <t>6 ventas de la región Norte alcanzaron la meta.</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="22" customHeight="1">
-      <c r="A8" s="2" t="inlineStr">
+    <row r="10" ht="28" customHeight="1">
+      <c r="A10" s="4" t="inlineStr">
         <is>
           <t>Laptop y Satisfacción &gt;=90%</t>
         </is>
       </c>
-      <c r="B8" s="3" t="inlineStr">
+      <c r="B10" s="5" t="inlineStr">
         <is>
           <t>CONTAR.SI.CONJUNTO()</t>
         </is>
       </c>
-      <c r="C8" s="4" t="n">
+      <c r="C10" s="6" t="n">
         <v>12</v>
       </c>
-      <c r="D8" s="2" t="inlineStr">
+      <c r="D10" s="4" t="inlineStr">
         <is>
           <t>12 ventas de Laptop tuvieron una satisfacción de 90% o más.</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="22" customHeight="1">
-      <c r="A9" s="5" t="inlineStr">
+    <row r="11" ht="28" customHeight="1">
+      <c r="A11" s="7" t="inlineStr">
         <is>
           <t>Sur y Devoluciones &gt;=3</t>
         </is>
       </c>
-      <c r="B9" s="6" t="inlineStr">
+      <c r="B11" s="8" t="inlineStr">
         <is>
           <t>CONTAR.SI.CONJUNTO()</t>
         </is>
       </c>
-      <c r="C9" s="7" t="n">
+      <c r="C11" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="D9" s="5" t="inlineStr">
+      <c r="D11" s="7" t="inlineStr">
         <is>
           <t>3 ventas de la región Sur tuvieron 3 o más devoluciones.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D9"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <mergeCells count="1">
+    <mergeCell ref="A1:D1"/>
+  </mergeCells>
+  <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
   <pageSetup orientation="landscape" paperSize="3" fitToHeight="1" fitToWidth="1"/>
-  <headerFooter>
-    <oddHeader>&amp;CHoja1</oddHeader>
-    <oddFooter/>
-    <evenHeader/>
-    <evenFooter/>
-    <firstHeader/>
-    <firstFooter/>
-  </headerFooter>
 </worksheet>
 </file>
</xml_diff>